<commit_message>
Corrida | SFE-FAEN | 2026-04-13 11:05:00.196406
</commit_message>
<xml_diff>
--- a/indicadores/SFE-FAEN_out.xlsx
+++ b/indicadores/SFE-FAEN_out.xlsx
@@ -98,13 +98,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">12/03/2026</t>
+    <t xml:space="preserve">13/04/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">arodriguez</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2147,7 +2147,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.0787073357065213</v>
+        <v>0.0795144079973077</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2205,7 +2205,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.0045019406457769</v>
+        <v>0.00456810282255729</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2275,7 +2275,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.195867781913834</v>
+        <v>0.203287010299679</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2305,7 +2305,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.309614724134518</v>
+        <v>0.279093353675291</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -26834,7 +26834,7 @@
         <v>514</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0327209462770437</v>
+        <v>-0.0312229617733219</v>
       </c>
     </row>
     <row r="6">
@@ -26842,7 +26842,7 @@
         <v>515</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.00897795750518476</v>
+        <v>-0.00843628096979432</v>
       </c>
     </row>
     <row r="7">
@@ -26850,7 +26850,7 @@
         <v>516</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0121297685983055</v>
+        <v>0.0116409638227243</v>
       </c>
     </row>
     <row r="8">
@@ -26858,7 +26858,7 @@
         <v>517</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.00232244267084745</v>
+        <v>0.00250824551781181</v>
       </c>
     </row>
     <row r="9">
@@ -26866,7 +26866,7 @@
         <v>518</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>-0.0204108436702082</v>
+        <v>-0.0201225815631736</v>
       </c>
     </row>
     <row r="10">
@@ -26874,7 +26874,7 @@
         <v>519</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>-0.041551320730114</v>
+        <v>-0.0426286301630395</v>
       </c>
     </row>
     <row r="11">
@@ -26882,7 +26882,7 @@
         <v>520</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>-0.0649763456134378</v>
+        <v>-0.0657512204186149</v>
       </c>
     </row>
     <row r="12">
@@ -26890,7 +26890,7 @@
         <v>521</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.0319029407720631</v>
+        <v>-0.0315446116563919</v>
       </c>
     </row>
     <row r="13">
@@ -26898,7 +26898,7 @@
         <v>522</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.0400069568680089</v>
+        <v>0.0405667021296851</v>
       </c>
     </row>
     <row r="14">
@@ -26906,7 +26906,7 @@
         <v>523</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.0670965024854269</v>
+        <v>0.0675877416589525</v>
       </c>
     </row>
     <row r="15">
@@ -26914,7 +26914,7 @@
         <v>524</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.0239958115408408</v>
+        <v>0.0244710100011334</v>
       </c>
     </row>
     <row r="16">
@@ -26922,7 +26922,7 @@
         <v>525</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>-0.0146338169465037</v>
+        <v>-0.0145822508141748</v>
       </c>
     </row>
     <row r="17">
@@ -26930,7 +26930,7 @@
         <v>526</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>-0.0386075591711137</v>
+        <v>-0.0398267648595219</v>
       </c>
     </row>
     <row r="18">
@@ -26938,7 +26938,7 @@
         <v>527</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>-0.0575666256924669</v>
+        <v>-0.0595480176077317</v>
       </c>
     </row>
     <row r="19">
@@ -26946,7 +26946,7 @@
         <v>528</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>-0.025740060619208</v>
+        <v>-0.0268190470909198</v>
       </c>
     </row>
     <row r="20">
@@ -26954,7 +26954,7 @@
         <v>529</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0135656091937005</v>
+        <v>0.0126800752122826</v>
       </c>
     </row>
     <row r="21">
@@ -26962,7 +26962,7 @@
         <v>530</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.0208295049636609</v>
+        <v>0.0199631673732437</v>
       </c>
     </row>
     <row r="22">
@@ -26970,7 +26970,7 @@
         <v>531</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.042088575217419</v>
+        <v>0.0424159950285569</v>
       </c>
     </row>
     <row r="23">
@@ -26978,7 +26978,7 @@
         <v>532</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.0787073357065213</v>
+        <v>0.0795144079973077</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-FAEN | 2026-05-12 10:58:46.270566
</commit_message>
<xml_diff>
--- a/indicadores/SFE-FAEN_out.xlsx
+++ b/indicadores/SFE-FAEN_out.xlsx
@@ -98,7 +98,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">13/04/2026</t>
+    <t xml:space="preserve">12/05/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -2147,7 +2147,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.0794008609780194</v>
+        <v>0.07910084493995</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2205,7 +2205,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.00456842219701286</v>
+        <v>0.00439119558655658</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2275,7 +2275,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.206115176192255</v>
+        <v>0.231443336795203</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2305,7 +2305,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.280275033958319</v>
+        <v>0.272685000792428</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -26870,7 +26870,7 @@
         <v>514</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.030357869488927</v>
+        <v>-0.0290523580395143</v>
       </c>
     </row>
     <row r="6">
@@ -26878,7 +26878,7 @@
         <v>515</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.00895411443722808</v>
+        <v>-0.00683978241019082</v>
       </c>
     </row>
     <row r="7">
@@ -26886,7 +26886,7 @@
         <v>516</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.0117865323618137</v>
+        <v>0.0112412456810021</v>
       </c>
     </row>
     <row r="8">
@@ -26894,7 +26894,7 @@
         <v>517</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.00299051600004883</v>
+        <v>0.00265556782964836</v>
       </c>
     </row>
     <row r="9">
@@ -26902,7 +26902,7 @@
         <v>518</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>-0.0205499546784649</v>
+        <v>-0.019291417226325</v>
       </c>
     </row>
     <row r="10">
@@ -26910,7 +26910,7 @@
         <v>519</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>-0.0424234603401948</v>
+        <v>-0.0434477591688248</v>
       </c>
     </row>
     <row r="11">
@@ -26918,7 +26918,7 @@
         <v>520</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>-0.0649221356793823</v>
+        <v>-0.0661386850331242</v>
       </c>
     </row>
     <row r="12">
@@ -26926,7 +26926,7 @@
         <v>521</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.0315695455003367</v>
+        <v>-0.0305564262646633</v>
       </c>
     </row>
     <row r="13">
@@ -26934,7 +26934,7 @@
         <v>522</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.0400665207073433</v>
+        <v>0.0402695713164509</v>
       </c>
     </row>
     <row r="14">
@@ -26942,7 +26942,7 @@
         <v>523</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.0675901042831926</v>
+        <v>0.0662660968109378</v>
       </c>
     </row>
     <row r="15">
@@ -26950,7 +26950,7 @@
         <v>524</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.0243264473713577</v>
+        <v>0.0241430359398577</v>
       </c>
     </row>
     <row r="16">
@@ -26958,7 +26958,7 @@
         <v>525</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>-0.0148527834167769</v>
+        <v>-0.0143377546373618</v>
       </c>
     </row>
     <row r="17">
@@ -26966,7 +26966,7 @@
         <v>526</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>-0.0400432818053357</v>
+        <v>-0.0396928002819423</v>
       </c>
     </row>
     <row r="18">
@@ -26974,7 +26974,7 @@
         <v>527</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>-0.0594645826068074</v>
+        <v>-0.0590201163176743</v>
       </c>
     </row>
     <row r="19">
@@ -26982,7 +26982,7 @@
         <v>528</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>-0.026667963100097</v>
+        <v>-0.0259969627933136</v>
       </c>
     </row>
     <row r="20">
@@ -26990,7 +26990,7 @@
         <v>529</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.0126752087564933</v>
+        <v>0.0128228127056993</v>
       </c>
     </row>
     <row r="21">
@@ -26998,7 +26998,7 @@
         <v>530</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.0198083759326795</v>
+        <v>0.0193001446960244</v>
       </c>
     </row>
     <row r="22">
@@ -27006,7 +27006,7 @@
         <v>531</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.0422214702789733</v>
+        <v>0.041871308407699</v>
       </c>
     </row>
     <row r="23">
@@ -27014,7 +27014,7 @@
         <v>532</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.0794008609780194</v>
+        <v>0.07910084493995</v>
       </c>
     </row>
     <row r="24">
@@ -27042,237 +27042,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2B3E1ED-F9B0-4FAD-879C-6F43AC0FA7C1}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F25231B6-5B33-4A3A-94C8-C6A9DE701749}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04F194D0-EBAC-4A91-AA12-0A662ECE7E1B}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-FAEN | 2026-06-08 11:27:08.300258
</commit_message>
<xml_diff>
--- a/indicadores/SFE-FAEN_out.xlsx
+++ b/indicadores/SFE-FAEN_out.xlsx
@@ -98,13 +98,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">12/05/2026</t>
+    <t xml:space="preserve">08/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">arodriguez</t>
+    <t xml:space="preserve">ysonder</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2147,7 +2147,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.0715541887896572</v>
+        <v>0.0730738880937111</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2205,7 +2205,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.00430598745041239</v>
+        <v>0.00455752405428116</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2275,7 +2275,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.24123553693545</v>
+        <v>0.262444291389116</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2305,7 +2305,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.579318151416861</v>
+        <v>0.666280413894853</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -26906,7 +26906,7 @@
         <v>514</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0308717255323404</v>
+        <v>-0.0285123508599751</v>
       </c>
     </row>
     <row r="6">
@@ -26914,7 +26914,7 @@
         <v>515</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.00601253758260633</v>
+        <v>-0.0061317816849028</v>
       </c>
     </row>
     <row r="7">
@@ -26922,7 +26922,7 @@
         <v>516</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.00503968697359259</v>
+        <v>-0.000415742623673726</v>
       </c>
     </row>
     <row r="8">
@@ -26930,7 +26930,7 @@
         <v>517</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.00617661087577585</v>
+        <v>0.00191082365340434</v>
       </c>
     </row>
     <row r="9">
@@ -26938,7 +26938,7 @@
         <v>518</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>-0.0071637574166181</v>
+        <v>-0.00427970913646018</v>
       </c>
     </row>
     <row r="10">
@@ -26946,7 +26946,7 @@
         <v>519</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>-0.0426223540763897</v>
+        <v>-0.0381420010600385</v>
       </c>
     </row>
     <row r="11">
@@ -26954,7 +26954,7 @@
         <v>520</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>-0.069794558543383</v>
+        <v>-0.0728408865410957</v>
       </c>
     </row>
     <row r="12">
@@ -26962,7 +26962,7 @@
         <v>521</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.0366114334813028</v>
+        <v>-0.0438174263686008</v>
       </c>
     </row>
     <row r="13">
@@ -26970,7 +26970,7 @@
         <v>522</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.0344576515850815</v>
+        <v>0.0313044141892028</v>
       </c>
     </row>
     <row r="14">
@@ -26978,7 +26978,7 @@
         <v>523</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.0656200232430041</v>
+        <v>0.0675094367794693</v>
       </c>
     </row>
     <row r="15">
@@ -26986,7 +26986,7 @@
         <v>524</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.0246039749331755</v>
+        <v>0.0287827444699326</v>
       </c>
     </row>
     <row r="16">
@@ -26994,7 +26994,7 @@
         <v>525</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>-0.0131228978358958</v>
+        <v>-0.00933556309444922</v>
       </c>
     </row>
     <row r="17">
@@ -27002,7 +27002,7 @@
         <v>526</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>-0.0301931085262194</v>
+        <v>-0.0273305408319265</v>
       </c>
     </row>
     <row r="18">
@@ -27010,7 +27010,7 @@
         <v>527</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>-0.0405496897303152</v>
+        <v>-0.038670021329736</v>
       </c>
     </row>
     <row r="19">
@@ -27018,7 +27018,7 @@
         <v>528</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>-0.00666269518245396</v>
+        <v>-0.00721645714684761</v>
       </c>
     </row>
     <row r="20">
@@ -27026,7 +27026,7 @@
         <v>529</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.023582913688762</v>
+        <v>0.020203526698983</v>
       </c>
     </row>
     <row r="21">
@@ -27034,7 +27034,7 @@
         <v>530</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.0138477307359059</v>
+        <v>0.0096707245313928</v>
       </c>
     </row>
     <row r="22">
@@ -27042,7 +27042,7 @@
         <v>531</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.0281420005426356</v>
+        <v>0.025965663071943</v>
       </c>
     </row>
     <row r="23">
@@ -27050,7 +27050,7 @@
         <v>532</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.0715541887896572</v>
+        <v>0.0730738880937111</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-FAEN | 2026-06-17 12:03:16.566733
</commit_message>
<xml_diff>
--- a/indicadores/SFE-FAEN_out.xlsx
+++ b/indicadores/SFE-FAEN_out.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="535" uniqueCount="535">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -23,7 +23,7 @@
     <t xml:space="preserve">Título</t>
   </si>
   <si>
-    <t xml:space="preserve">Faena bovina, porcina y aviar en la provincia de Santa Fe</t>
+    <t xml:space="preserve">Faena bovina, porcina y aviar</t>
   </si>
   <si>
     <t xml:space="preserve">Unidad de medida</t>
@@ -65,6 +65,12 @@
     <t xml:space="preserve">Regresores</t>
   </si>
   <si>
+    <t xml:space="preserve">Alcance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provincia de Santa Fe</t>
+  </si>
+  <si>
     <t xml:space="preserve">Resumen del correlograma</t>
   </si>
   <si>
@@ -98,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">08/06/2026</t>
+    <t xml:space="preserve">17/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">ysonder</t>
+    <t xml:space="preserve">focampo</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2115,9 +2121,13 @@
       <c r="J6" s="1"/>
     </row>
     <row r="7">
-      <c r="A7"/>
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
       <c r="B7"/>
-      <c r="C7"/>
+      <c r="C7" t="s">
+        <v>17</v>
+      </c>
       <c r="D7"/>
       <c r="E7"/>
       <c r="F7"/>
@@ -2128,7 +2138,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8"/>
       <c r="C8"/>
@@ -2142,7 +2152,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B9"/>
       <c r="C9"/>
@@ -2158,7 +2168,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B10"/>
       <c r="C10"/>
@@ -2186,7 +2196,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B12"/>
       <c r="C12"/>
@@ -2200,7 +2210,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B13"/>
       <c r="C13"/>
@@ -2228,7 +2238,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B15"/>
       <c r="C15"/>
@@ -2242,7 +2252,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B16"/>
       <c r="C16"/>
@@ -2256,7 +2266,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B17"/>
       <c r="C17"/>
@@ -2270,7 +2280,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B18"/>
       <c r="C18"/>
@@ -2286,7 +2296,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B19"/>
       <c r="C19"/>
@@ -2300,7 +2310,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B20"/>
       <c r="C20"/>
@@ -2448,10 +2458,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B32" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C32"/>
       <c r="D32"/>
@@ -2464,10 +2474,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B33" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C33"/>
       <c r="D33"/>
@@ -2491,66 +2501,66 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C1" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E1" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G1" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H1" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I1" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J1" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K1" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="L1" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="M1" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N1" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="O1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="P1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="Q1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="R1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="S1" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B2" s="2" t="n">
         <v>41981.4179124854</v>
@@ -2603,7 +2613,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B3" s="2" t="n">
         <v>40004.135575284</v>
@@ -2660,7 +2670,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B4" s="2" t="n">
         <v>46407.9650305985</v>
@@ -2717,7 +2727,7 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B5" s="2" t="n">
         <v>41971.1454685882</v>
@@ -2774,7 +2784,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B6" s="2" t="n">
         <v>45187.7263970581</v>
@@ -2831,7 +2841,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B7" s="2" t="n">
         <v>44586.9202087399</v>
@@ -2888,7 +2898,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B8" s="2" t="n">
         <v>44657.3293516836</v>
@@ -2945,7 +2955,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B9" s="2" t="n">
         <v>47026.665789164</v>
@@ -3002,7 +3012,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B10" s="2" t="n">
         <v>48077.4894589629</v>
@@ -3059,7 +3069,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B11" s="2" t="n">
         <v>47534.4007253003</v>
@@ -3116,7 +3126,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B12" s="2" t="n">
         <v>50814.5854104873</v>
@@ -3173,7 +3183,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B13" s="2" t="n">
         <v>49535.3794049399</v>
@@ -3230,7 +3240,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B14" s="2" t="n">
         <v>50214.4429574218</v>
@@ -3289,7 +3299,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B15" s="2" t="n">
         <v>47857.1530786041</v>
@@ -3348,7 +3358,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>55017.3500581094</v>
@@ -3407,7 +3417,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B17" s="2" t="n">
         <v>47087.6537588076</v>
@@ -3466,7 +3476,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B18" s="2" t="n">
         <v>54058.9748649081</v>
@@ -3525,7 +3535,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B19" s="2" t="n">
         <v>53172.149669894</v>
@@ -3584,7 +3594,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B20" s="2" t="n">
         <v>51472.7351199625</v>
@@ -3643,7 +3653,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B21" s="2" t="n">
         <v>55278.8261289747</v>
@@ -3702,7 +3712,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B22" s="2" t="n">
         <v>51312.2434916873</v>
@@ -3761,7 +3771,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B23" s="2" t="n">
         <v>49051.467371917</v>
@@ -3820,7 +3830,7 @@
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B24" s="2" t="n">
         <v>51024.1398911554</v>
@@ -3879,7 +3889,7 @@
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B25" s="2" t="n">
         <v>45840.4114195814</v>
@@ -3938,7 +3948,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B26" s="2" t="n">
         <v>51930.6155113786</v>
@@ -3997,7 +4007,7 @@
     </row>
     <row r="27">
       <c r="A27" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B27" s="2" t="n">
         <v>50510.9646915482</v>
@@ -4056,7 +4066,7 @@
     </row>
     <row r="28">
       <c r="A28" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B28" s="2" t="n">
         <v>52007.7214181319</v>
@@ -4115,7 +4125,7 @@
     </row>
     <row r="29">
       <c r="A29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B29" s="2" t="n">
         <v>50160.907661074</v>
@@ -4174,7 +4184,7 @@
     </row>
     <row r="30">
       <c r="A30" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B30" s="2" t="n">
         <v>50565.6603375587</v>
@@ -4233,7 +4243,7 @@
     </row>
     <row r="31">
       <c r="A31" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B31" s="2" t="n">
         <v>45825.8925764022</v>
@@ -4292,7 +4302,7 @@
     </row>
     <row r="32">
       <c r="A32" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B32" s="2" t="n">
         <v>51759.8243758377</v>
@@ -4351,7 +4361,7 @@
     </row>
     <row r="33">
       <c r="A33" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B33" s="2" t="n">
         <v>50558.5001623564</v>
@@ -4410,7 +4420,7 @@
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B34" s="2" t="n">
         <v>48336.1725476757</v>
@@ -4469,7 +4479,7 @@
     </row>
     <row r="35">
       <c r="A35" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B35" s="2" t="n">
         <v>52968.9331204161</v>
@@ -4528,7 +4538,7 @@
     </row>
     <row r="36">
       <c r="A36" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B36" s="2" t="n">
         <v>50017.4532179504</v>
@@ -4587,7 +4597,7 @@
     </row>
     <row r="37">
       <c r="A37" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B37" s="2" t="n">
         <v>48902.9964125369</v>
@@ -4646,7 +4656,7 @@
     </row>
     <row r="38">
       <c r="A38" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B38" s="2" t="n">
         <v>51482.3426580715</v>
@@ -4705,7 +4715,7 @@
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B39" s="2" t="n">
         <v>48894.4914705517</v>
@@ -4764,7 +4774,7 @@
     </row>
     <row r="40">
       <c r="A40" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B40" s="2" t="n">
         <v>50736.9353128686</v>
@@ -4823,7 +4833,7 @@
     </row>
     <row r="41">
       <c r="A41" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B41" s="2" t="n">
         <v>57894.8033649995</v>
@@ -4882,7 +4892,7 @@
     </row>
     <row r="42">
       <c r="A42" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B42" s="2" t="n">
         <v>56975.9246663259</v>
@@ -4941,7 +4951,7 @@
     </row>
     <row r="43">
       <c r="A43" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B43" s="2" t="n">
         <v>52979.4089175772</v>
@@ -5000,7 +5010,7 @@
     </row>
     <row r="44">
       <c r="A44" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B44" s="2" t="n">
         <v>53428.9812914575</v>
@@ -5059,7 +5069,7 @@
     </row>
     <row r="45">
       <c r="A45" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B45" s="2" t="n">
         <v>47793.6154877182</v>
@@ -5118,7 +5128,7 @@
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B46" s="2" t="n">
         <v>50147.5644514484</v>
@@ -5177,7 +5187,7 @@
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B47" s="2" t="n">
         <v>48328.1071957389</v>
@@ -5236,7 +5246,7 @@
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B48" s="2" t="n">
         <v>43871.1839872458</v>
@@ -5295,7 +5305,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B49" s="2" t="n">
         <v>45948.2838717172</v>
@@ -5354,7 +5364,7 @@
     </row>
     <row r="50">
       <c r="A50" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B50" s="2" t="n">
         <v>46185.5691230028</v>
@@ -5413,7 +5423,7 @@
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B51" s="2" t="n">
         <v>40768.2112801119</v>
@@ -5472,7 +5482,7 @@
     </row>
     <row r="52">
       <c r="A52" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B52" s="2" t="n">
         <v>46775.0822509864</v>
@@ -5531,7 +5541,7 @@
     </row>
     <row r="53">
       <c r="A53" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B53" s="2" t="n">
         <v>45571.6971193792</v>
@@ -5590,7 +5600,7 @@
     </row>
     <row r="54">
       <c r="A54" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B54" s="2" t="n">
         <v>44492.0353589814</v>
@@ -5649,7 +5659,7 @@
     </row>
     <row r="55">
       <c r="A55" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B55" s="2" t="n">
         <v>42859.2913238547</v>
@@ -5708,7 +5718,7 @@
     </row>
     <row r="56">
       <c r="A56" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B56" s="2" t="n">
         <v>41565.2392814377</v>
@@ -5767,7 +5777,7 @@
     </row>
     <row r="57">
       <c r="A57" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B57" s="2" t="n">
         <v>42060.645344716</v>
@@ -5826,7 +5836,7 @@
     </row>
     <row r="58">
       <c r="A58" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B58" s="2" t="n">
         <v>47342.9163041894</v>
@@ -5885,7 +5895,7 @@
     </row>
     <row r="59">
       <c r="A59" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B59" s="2" t="n">
         <v>48467.8763189009</v>
@@ -5944,7 +5954,7 @@
     </row>
     <row r="60">
       <c r="A60" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B60" s="2" t="n">
         <v>49486.9384527977</v>
@@ -6003,7 +6013,7 @@
     </row>
     <row r="61">
       <c r="A61" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B61" s="2" t="n">
         <v>50263.4686298846</v>
@@ -6062,7 +6072,7 @@
     </row>
     <row r="62">
       <c r="A62" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B62" s="2" t="n">
         <v>49405.4098938183</v>
@@ -6121,7 +6131,7 @@
     </row>
     <row r="63">
       <c r="A63" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B63" s="2" t="n">
         <v>44507.0579128051</v>
@@ -6180,7 +6190,7 @@
     </row>
     <row r="64">
       <c r="A64" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B64" s="2" t="n">
         <v>49654.0311076638</v>
@@ -6239,7 +6249,7 @@
     </row>
     <row r="65">
       <c r="A65" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B65" s="2" t="n">
         <v>45872.7349663773</v>
@@ -6298,7 +6308,7 @@
     </row>
     <row r="66">
       <c r="A66" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B66" s="2" t="n">
         <v>48333.3156940389</v>
@@ -6357,7 +6367,7 @@
     </row>
     <row r="67">
       <c r="A67" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B67" s="2" t="n">
         <v>46097.1031056252</v>
@@ -6416,7 +6426,7 @@
     </row>
     <row r="68">
       <c r="A68" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B68" s="2" t="n">
         <v>45522.53790453</v>
@@ -6475,7 +6485,7 @@
     </row>
     <row r="69">
       <c r="A69" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B69" s="2" t="n">
         <v>47192.6434833162</v>
@@ -6534,7 +6544,7 @@
     </row>
     <row r="70">
       <c r="A70" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B70" s="2" t="n">
         <v>48782.5576338529</v>
@@ -6593,7 +6603,7 @@
     </row>
     <row r="71">
       <c r="A71" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B71" s="2" t="n">
         <v>48060.488464815</v>
@@ -6652,7 +6662,7 @@
     </row>
     <row r="72">
       <c r="A72" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B72" s="2" t="n">
         <v>52329.6455068009</v>
@@ -6711,7 +6721,7 @@
     </row>
     <row r="73">
       <c r="A73" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B73" s="2" t="n">
         <v>50222.6514802075</v>
@@ -6770,7 +6780,7 @@
     </row>
     <row r="74">
       <c r="A74" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B74" s="2" t="n">
         <v>49297.1937410586</v>
@@ -6829,7 +6839,7 @@
     </row>
     <row r="75">
       <c r="A75" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B75" s="2" t="n">
         <v>46270.5221452188</v>
@@ -6888,7 +6898,7 @@
     </row>
     <row r="76">
       <c r="A76" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B76" s="2" t="n">
         <v>51621.2231914298</v>
@@ -6947,7 +6957,7 @@
     </row>
     <row r="77">
       <c r="A77" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B77" s="2" t="n">
         <v>41958.0595518639</v>
@@ -7006,7 +7016,7 @@
     </row>
     <row r="78">
       <c r="A78" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B78" s="2" t="n">
         <v>47838.6304931878</v>
@@ -7065,7 +7075,7 @@
     </row>
     <row r="79">
       <c r="A79" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B79" s="2" t="n">
         <v>47734.2214277444</v>
@@ -7124,7 +7134,7 @@
     </row>
     <row r="80">
       <c r="A80" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B80" s="2" t="n">
         <v>47969.2193323875</v>
@@ -7183,7 +7193,7 @@
     </row>
     <row r="81">
       <c r="A81" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B81" s="2" t="n">
         <v>45460.8716709334</v>
@@ -7242,7 +7252,7 @@
     </row>
     <row r="82">
       <c r="A82" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B82" s="2" t="n">
         <v>46484.9662904542</v>
@@ -7301,7 +7311,7 @@
     </row>
     <row r="83">
       <c r="A83" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B83" s="2" t="n">
         <v>44569.3066417887</v>
@@ -7360,7 +7370,7 @@
     </row>
     <row r="84">
       <c r="A84" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B84" s="2" t="n">
         <v>46227.9659031895</v>
@@ -7419,7 +7429,7 @@
     </row>
     <row r="85">
       <c r="A85" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B85" s="2" t="n">
         <v>44913.8888634898</v>
@@ -7478,7 +7488,7 @@
     </row>
     <row r="86">
       <c r="A86" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B86" s="2" t="n">
         <v>45558.8784511376</v>
@@ -7537,7 +7547,7 @@
     </row>
     <row r="87">
       <c r="A87" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B87" s="2" t="n">
         <v>42110.1255094064</v>
@@ -7596,7 +7606,7 @@
     </row>
     <row r="88">
       <c r="A88" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B88" s="2" t="n">
         <v>37776.1445155091</v>
@@ -7655,7 +7665,7 @@
     </row>
     <row r="89">
       <c r="A89" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B89" s="2" t="n">
         <v>34926.1480687087</v>
@@ -7714,7 +7724,7 @@
     </row>
     <row r="90">
       <c r="A90" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B90" s="2" t="n">
         <v>37625.5128336015</v>
@@ -7773,7 +7783,7 @@
     </row>
     <row r="91">
       <c r="A91" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B91" s="2" t="n">
         <v>36799.5387699925</v>
@@ -7832,7 +7842,7 @@
     </row>
     <row r="92">
       <c r="A92" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B92" s="2" t="n">
         <v>39205.1935815453</v>
@@ -7891,7 +7901,7 @@
     </row>
     <row r="93">
       <c r="A93" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B93" s="2" t="n">
         <v>39548.6530095455</v>
@@ -7950,7 +7960,7 @@
     </row>
     <row r="94">
       <c r="A94" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B94" s="2" t="n">
         <v>35795.749515432</v>
@@ -8009,7 +8019,7 @@
     </row>
     <row r="95">
       <c r="A95" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B95" s="2" t="n">
         <v>40560.9265610725</v>
@@ -8068,7 +8078,7 @@
     </row>
     <row r="96">
       <c r="A96" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B96" s="2" t="n">
         <v>39249.170543493</v>
@@ -8127,7 +8137,7 @@
     </row>
     <row r="97">
       <c r="A97" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B97" s="2" t="n">
         <v>37129.569161281</v>
@@ -8186,7 +8196,7 @@
     </row>
     <row r="98">
       <c r="A98" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B98" s="2" t="n">
         <v>35159.3362819959</v>
@@ -8245,7 +8255,7 @@
     </row>
     <row r="99">
       <c r="A99" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B99" s="2" t="n">
         <v>38112.9898472697</v>
@@ -8304,7 +8314,7 @@
     </row>
     <row r="100">
       <c r="A100" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B100" s="2" t="n">
         <v>41949.7466532123</v>
@@ -8363,7 +8373,7 @@
     </row>
     <row r="101">
       <c r="A101" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B101" s="2" t="n">
         <v>43064.9928950521</v>
@@ -8422,7 +8432,7 @@
     </row>
     <row r="102">
       <c r="A102" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B102" s="2" t="n">
         <v>45767.1610093191</v>
@@ -8481,7 +8491,7 @@
     </row>
     <row r="103">
       <c r="A103" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B103" s="2" t="n">
         <v>46685.4987898702</v>
@@ -8540,7 +8550,7 @@
     </row>
     <row r="104">
       <c r="A104" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B104" s="2" t="n">
         <v>48091.588016277</v>
@@ -8599,7 +8609,7 @@
     </row>
     <row r="105">
       <c r="A105" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B105" s="2" t="n">
         <v>45165.0583570739</v>
@@ -8658,7 +8668,7 @@
     </row>
     <row r="106">
       <c r="A106" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B106" s="2" t="n">
         <v>42808.0235377069</v>
@@ -8717,7 +8727,7 @@
     </row>
     <row r="107">
       <c r="A107" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B107" s="2" t="n">
         <v>43983.3241920523</v>
@@ -8776,7 +8786,7 @@
     </row>
     <row r="108">
       <c r="A108" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B108" s="2" t="n">
         <v>44008.0801290528</v>
@@ -8835,7 +8845,7 @@
     </row>
     <row r="109">
       <c r="A109" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B109" s="2" t="n">
         <v>41301.6250868543</v>
@@ -8894,7 +8904,7 @@
     </row>
     <row r="110">
       <c r="A110" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B110" s="2" t="n">
         <v>44439.4741083941</v>
@@ -8953,7 +8963,7 @@
     </row>
     <row r="111">
       <c r="A111" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B111" s="2" t="n">
         <v>38124.8922350339</v>
@@ -9012,7 +9022,7 @@
     </row>
     <row r="112">
       <c r="A112" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B112" s="2" t="n">
         <v>41106.5543618564</v>
@@ -9071,7 +9081,7 @@
     </row>
     <row r="113">
       <c r="A113" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B113" s="2" t="n">
         <v>40082.0626914384</v>
@@ -9130,7 +9140,7 @@
     </row>
     <row r="114">
       <c r="A114" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B114" s="2" t="n">
         <v>41271.4604601594</v>
@@ -9189,7 +9199,7 @@
     </row>
     <row r="115">
       <c r="A115" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B115" s="2" t="n">
         <v>44620.8303899069</v>
@@ -9248,7 +9258,7 @@
     </row>
     <row r="116">
       <c r="A116" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B116" s="2" t="n">
         <v>50042.757012091</v>
@@ -9307,7 +9317,7 @@
     </row>
     <row r="117">
       <c r="A117" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B117" s="2" t="n">
         <v>45711.52410049</v>
@@ -9366,7 +9376,7 @@
     </row>
     <row r="118">
       <c r="A118" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B118" s="2" t="n">
         <v>49220.1181950956</v>
@@ -9425,7 +9435,7 @@
     </row>
     <row r="119">
       <c r="A119" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B119" s="2" t="n">
         <v>51153.8008652069</v>
@@ -9484,7 +9494,7 @@
     </row>
     <row r="120">
       <c r="A120" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B120" s="2" t="n">
         <v>50596.1281253808</v>
@@ -9543,7 +9553,7 @@
     </row>
     <row r="121">
       <c r="A121" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B121" s="2" t="n">
         <v>52005.6092528917</v>
@@ -9602,7 +9612,7 @@
     </row>
     <row r="122">
       <c r="A122" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B122" s="2" t="n">
         <v>50186.0403918062</v>
@@ -9661,7 +9671,7 @@
     </row>
     <row r="123">
       <c r="A123" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B123" s="2" t="n">
         <v>48045.9806403483</v>
@@ -9720,7 +9730,7 @@
     </row>
     <row r="124">
       <c r="A124" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B124" s="2" t="n">
         <v>55639.4743089379</v>
@@ -9779,7 +9789,7 @@
     </row>
     <row r="125">
       <c r="A125" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B125" s="2" t="n">
         <v>47389.0108738654</v>
@@ -9838,7 +9848,7 @@
     </row>
     <row r="126">
       <c r="A126" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B126" s="2" t="n">
         <v>51124.5484448688</v>
@@ -9897,7 +9907,7 @@
     </row>
     <row r="127">
       <c r="A127" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B127" s="2" t="n">
         <v>55636.8327020116</v>
@@ -9956,7 +9966,7 @@
     </row>
     <row r="128">
       <c r="A128" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B128" s="2" t="n">
         <v>55982.8352252656</v>
@@ -10015,7 +10025,7 @@
     </row>
     <row r="129">
       <c r="A129" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B129" s="2" t="n">
         <v>54787.4516058734</v>
@@ -10074,7 +10084,7 @@
     </row>
     <row r="130">
       <c r="A130" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B130" s="2" t="n">
         <v>58205.5901951777</v>
@@ -10133,7 +10143,7 @@
     </row>
     <row r="131">
       <c r="A131" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B131" s="2" t="n">
         <v>56494.2452863137</v>
@@ -10192,7 +10202,7 @@
     </row>
     <row r="132">
       <c r="A132" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B132" s="2" t="n">
         <v>58624.6465463756</v>
@@ -10251,7 +10261,7 @@
     </row>
     <row r="133">
       <c r="A133" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B133" s="2" t="n">
         <v>56263.7074986155</v>
@@ -10310,7 +10320,7 @@
     </row>
     <row r="134">
       <c r="A134" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B134" s="2" t="n">
         <v>54790.1136015271</v>
@@ -10369,7 +10379,7 @@
     </row>
     <row r="135">
       <c r="A135" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B135" s="2" t="n">
         <v>52171.7922334838</v>
@@ -10428,7 +10438,7 @@
     </row>
     <row r="136">
       <c r="A136" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B136" s="2" t="n">
         <v>51614.1435265794</v>
@@ -10487,7 +10497,7 @@
     </row>
     <row r="137">
       <c r="A137" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B137" s="2" t="n">
         <v>54928.239634945</v>
@@ -10546,7 +10556,7 @@
     </row>
     <row r="138">
       <c r="A138" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B138" s="2" t="n">
         <v>53957.7009930532</v>
@@ -10605,7 +10615,7 @@
     </row>
     <row r="139">
       <c r="A139" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B139" s="2" t="n">
         <v>55184.2234917893</v>
@@ -10664,7 +10674,7 @@
     </row>
     <row r="140">
       <c r="A140" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B140" s="2" t="n">
         <v>55020.6448560658</v>
@@ -10723,7 +10733,7 @@
     </row>
     <row r="141">
       <c r="A141" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B141" s="2" t="n">
         <v>59702.7855576246</v>
@@ -10782,7 +10792,7 @@
     </row>
     <row r="142">
       <c r="A142" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B142" s="2" t="n">
         <v>57570.6638826455</v>
@@ -10841,7 +10851,7 @@
     </row>
     <row r="143">
       <c r="A143" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B143" s="2" t="n">
         <v>56608.2297049393</v>
@@ -10900,7 +10910,7 @@
     </row>
     <row r="144">
       <c r="A144" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B144" s="2" t="n">
         <v>58147.0774109152</v>
@@ -10959,7 +10969,7 @@
     </row>
     <row r="145">
       <c r="A145" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B145" s="2" t="n">
         <v>55753.9177518071</v>
@@ -11018,7 +11028,7 @@
     </row>
     <row r="146">
       <c r="A146" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B146" s="2" t="n">
         <v>54838.7624264546</v>
@@ -11077,7 +11087,7 @@
     </row>
     <row r="147">
       <c r="A147" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B147" s="2" t="n">
         <v>48329.1280634091</v>
@@ -11136,7 +11146,7 @@
     </row>
     <row r="148">
       <c r="A148" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B148" s="2" t="n">
         <v>53839.1127269179</v>
@@ -11195,7 +11205,7 @@
     </row>
     <row r="149">
       <c r="A149" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="B149" s="2" t="n">
         <v>40693.536618475</v>
@@ -11254,7 +11264,7 @@
     </row>
     <row r="150">
       <c r="A150" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B150" s="2" t="n">
         <v>45270.0293017328</v>
@@ -11313,7 +11323,7 @@
     </row>
     <row r="151">
       <c r="A151" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="B151" s="2" t="n">
         <v>51911.2276571706</v>
@@ -11372,7 +11382,7 @@
     </row>
     <row r="152">
       <c r="A152" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B152" s="2" t="n">
         <v>54266.7996334381</v>
@@ -11431,7 +11441,7 @@
     </row>
     <row r="153">
       <c r="A153" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B153" s="2" t="n">
         <v>59575.7352916188</v>
@@ -11490,7 +11500,7 @@
     </row>
     <row r="154">
       <c r="A154" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B154" s="2" t="n">
         <v>59284.8838255919</v>
@@ -11549,7 +11559,7 @@
     </row>
     <row r="155">
       <c r="A155" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B155" s="2" t="n">
         <v>57817.3041618744</v>
@@ -11608,7 +11618,7 @@
     </row>
     <row r="156">
       <c r="A156" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="B156" s="2" t="n">
         <v>58762.3832790036</v>
@@ -11667,7 +11677,7 @@
     </row>
     <row r="157">
       <c r="A157" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B157" s="2" t="n">
         <v>47036.6285329717</v>
@@ -11726,7 +11736,7 @@
     </row>
     <row r="158">
       <c r="A158" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B158" s="2" t="n">
         <v>57281.9842300777</v>
@@ -11785,7 +11795,7 @@
     </row>
     <row r="159">
       <c r="A159" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B159" s="2" t="n">
         <v>49644.3825864743</v>
@@ -11844,7 +11854,7 @@
     </row>
     <row r="160">
       <c r="A160" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B160" s="2" t="n">
         <v>53207.949792296</v>
@@ -11903,7 +11913,7 @@
     </row>
     <row r="161">
       <c r="A161" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B161" s="2" t="n">
         <v>50212.022806283</v>
@@ -11962,7 +11972,7 @@
     </row>
     <row r="162">
       <c r="A162" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="B162" s="2" t="n">
         <v>57547.7889053769</v>
@@ -12021,7 +12031,7 @@
     </row>
     <row r="163">
       <c r="A163" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B163" s="2" t="n">
         <v>56507.2491155936</v>
@@ -12080,7 +12090,7 @@
     </row>
     <row r="164">
       <c r="A164" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B164" s="2" t="n">
         <v>60919.4712574951</v>
@@ -12139,7 +12149,7 @@
     </row>
     <row r="165">
       <c r="A165" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B165" s="2" t="n">
         <v>63190.2844890024</v>
@@ -12198,7 +12208,7 @@
     </row>
     <row r="166">
       <c r="A166" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B166" s="2" t="n">
         <v>51313.7922232925</v>
@@ -12257,7 +12267,7 @@
     </row>
     <row r="167">
       <c r="A167" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="B167" s="2" t="n">
         <v>60329.8965981207</v>
@@ -12316,7 +12326,7 @@
     </row>
     <row r="168">
       <c r="A168" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B168" s="2" t="n">
         <v>65667.7219115512</v>
@@ -12375,7 +12385,7 @@
     </row>
     <row r="169">
       <c r="A169" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B169" s="2" t="n">
         <v>55864.6033069512</v>
@@ -12434,7 +12444,7 @@
     </row>
     <row r="170">
       <c r="A170" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B170" s="2" t="n">
         <v>59595.4316683233</v>
@@ -12493,7 +12503,7 @@
     </row>
     <row r="171">
       <c r="A171" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B171" s="2" t="n">
         <v>55240.5087666458</v>
@@ -12552,7 +12562,7 @@
     </row>
     <row r="172">
       <c r="A172" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B172" s="2" t="n">
         <v>35377.6076535416</v>
@@ -12611,7 +12621,7 @@
     </row>
     <row r="173">
       <c r="A173" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B173" s="2" t="n">
         <v>57229.2124409121</v>
@@ -12670,7 +12680,7 @@
     </row>
     <row r="174">
       <c r="A174" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B174" s="2" t="n">
         <v>46405.928221517</v>
@@ -12729,7 +12739,7 @@
     </row>
     <row r="175">
       <c r="A175" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B175" s="2" t="n">
         <v>42989.8673191694</v>
@@ -12788,7 +12798,7 @@
     </row>
     <row r="176">
       <c r="A176" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="B176" s="2" t="n">
         <v>66286.9552458859</v>
@@ -12847,7 +12857,7 @@
     </row>
     <row r="177">
       <c r="A177" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B177" s="2" t="n">
         <v>62407.2088602623</v>
@@ -12906,7 +12916,7 @@
     </row>
     <row r="178">
       <c r="A178" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B178" s="2" t="n">
         <v>64528.0048623493</v>
@@ -12965,7 +12975,7 @@
     </row>
     <row r="179">
       <c r="A179" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B179" s="2" t="n">
         <v>57312.6721329333</v>
@@ -13024,7 +13034,7 @@
     </row>
     <row r="180">
       <c r="A180" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B180" s="2" t="n">
         <v>53581.0634634365</v>
@@ -13083,7 +13093,7 @@
     </row>
     <row r="181">
       <c r="A181" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B181" s="2" t="n">
         <v>53286.3173427846</v>
@@ -13142,7 +13152,7 @@
     </row>
     <row r="182">
       <c r="A182" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B182" s="2" t="n">
         <v>56733.4369327775</v>
@@ -13201,7 +13211,7 @@
     </row>
     <row r="183">
       <c r="A183" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B183" s="2" t="n">
         <v>52415.2283738553</v>
@@ -13260,7 +13270,7 @@
     </row>
     <row r="184">
       <c r="A184" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B184" s="2" t="n">
         <v>54974.2417110417</v>
@@ -13319,7 +13329,7 @@
     </row>
     <row r="185">
       <c r="A185" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B185" s="2" t="n">
         <v>59416.0166856611</v>
@@ -13378,7 +13388,7 @@
     </row>
     <row r="186">
       <c r="A186" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B186" s="2" t="n">
         <v>56507.0811189922</v>
@@ -13437,7 +13447,7 @@
     </row>
     <row r="187">
       <c r="A187" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="B187" s="2" t="n">
         <v>64070.3522643093</v>
@@ -13496,7 +13506,7 @@
     </row>
     <row r="188">
       <c r="A188" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="B188" s="2" t="n">
         <v>65139.9202497621</v>
@@ -13555,7 +13565,7 @@
     </row>
     <row r="189">
       <c r="A189" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B189" s="2" t="n">
         <v>61466.8643385718</v>
@@ -13614,7 +13624,7 @@
     </row>
     <row r="190">
       <c r="A190" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="B190" s="2" t="n">
         <v>57277.1985408374</v>
@@ -13673,7 +13683,7 @@
     </row>
     <row r="191">
       <c r="A191" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B191" s="2" t="n">
         <v>64326.1578366066</v>
@@ -13732,7 +13742,7 @@
     </row>
     <row r="192">
       <c r="A192" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B192" s="2" t="n">
         <v>55529.3782582141</v>
@@ -13791,7 +13801,7 @@
     </row>
     <row r="193">
       <c r="A193" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="B193" s="2" t="n">
         <v>52759.1848800311</v>
@@ -13850,7 +13860,7 @@
     </row>
     <row r="194">
       <c r="A194" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B194" s="2" t="n">
         <v>50498.4984421436</v>
@@ -13909,7 +13919,7 @@
     </row>
     <row r="195">
       <c r="A195" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="B195" s="2" t="n">
         <v>46297.9772110204</v>
@@ -13968,7 +13978,7 @@
     </row>
     <row r="196">
       <c r="A196" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B196" s="2" t="n">
         <v>51119.8250432896</v>
@@ -14027,7 +14037,7 @@
     </row>
     <row r="197">
       <c r="A197" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B197" s="2" t="n">
         <v>46353.5366441657</v>
@@ -14086,7 +14096,7 @@
     </row>
     <row r="198">
       <c r="A198" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B198" s="2" t="n">
         <v>47608.9418517179</v>
@@ -14145,7 +14155,7 @@
     </row>
     <row r="199">
       <c r="A199" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B199" s="2" t="n">
         <v>47165.5673821432</v>
@@ -14204,7 +14214,7 @@
     </row>
     <row r="200">
       <c r="A200" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B200" s="2" t="n">
         <v>49803.4981511301</v>
@@ -14263,7 +14273,7 @@
     </row>
     <row r="201">
       <c r="A201" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="B201" s="2" t="n">
         <v>52373.2912195908</v>
@@ -14322,7 +14332,7 @@
     </row>
     <row r="202">
       <c r="A202" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B202" s="2" t="n">
         <v>48563.6829544301</v>
@@ -14381,7 +14391,7 @@
     </row>
     <row r="203">
       <c r="A203" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B203" s="2" t="n">
         <v>44346.9529943403</v>
@@ -14440,7 +14450,7 @@
     </row>
     <row r="204">
       <c r="A204" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B204" s="2" t="n">
         <v>48106.9012850882</v>
@@ -14499,7 +14509,7 @@
     </row>
     <row r="205">
       <c r="A205" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B205" s="2" t="n">
         <v>45037.9123291614</v>
@@ -14558,7 +14568,7 @@
     </row>
     <row r="206">
       <c r="A206" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B206" s="2" t="n">
         <v>42936.3887770468</v>
@@ -14617,7 +14627,7 @@
     </row>
     <row r="207">
       <c r="A207" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B207" s="2" t="n">
         <v>42896.8365634893</v>
@@ -14676,7 +14686,7 @@
     </row>
     <row r="208">
       <c r="A208" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B208" s="2" t="n">
         <v>47899.2607280539</v>
@@ -14735,7 +14745,7 @@
     </row>
     <row r="209">
       <c r="A209" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B209" s="2" t="n">
         <v>45702.7683287515</v>
@@ -14794,7 +14804,7 @@
     </row>
     <row r="210">
       <c r="A210" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B210" s="2" t="n">
         <v>49064.1712728148</v>
@@ -14853,7 +14863,7 @@
     </row>
     <row r="211">
       <c r="A211" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="B211" s="2" t="n">
         <v>47172.5765397591</v>
@@ -14912,7 +14922,7 @@
     </row>
     <row r="212">
       <c r="A212" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B212" s="2" t="n">
         <v>45334.9652937877</v>
@@ -14971,7 +14981,7 @@
     </row>
     <row r="213">
       <c r="A213" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B213" s="2" t="n">
         <v>49574.3460867543</v>
@@ -15030,7 +15040,7 @@
     </row>
     <row r="214">
       <c r="A214" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B214" s="2" t="n">
         <v>51088.2768526694</v>
@@ -15089,7 +15099,7 @@
     </row>
     <row r="215">
       <c r="A215" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B215" s="2" t="n">
         <v>47069.4070566806</v>
@@ -15148,7 +15158,7 @@
     </row>
     <row r="216">
       <c r="A216" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="B216" s="2" t="n">
         <v>46718.141557604</v>
@@ -15207,7 +15217,7 @@
     </row>
     <row r="217">
       <c r="A217" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B217" s="2" t="n">
         <v>46154.7681976744</v>
@@ -15266,7 +15276,7 @@
     </row>
     <row r="218">
       <c r="A218" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B218" s="2" t="n">
         <v>40764.6269146094</v>
@@ -15325,7 +15335,7 @@
     </row>
     <row r="219">
       <c r="A219" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B219" s="2" t="n">
         <v>36448.0014579212</v>
@@ -15384,7 +15394,7 @@
     </row>
     <row r="220">
       <c r="A220" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="B220" s="2" t="n">
         <v>52132.9913935795</v>
@@ -15443,7 +15453,7 @@
     </row>
     <row r="221">
       <c r="A221" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B221" s="2" t="n">
         <v>47326.8685848688</v>
@@ -15502,7 +15512,7 @@
     </row>
     <row r="222">
       <c r="A222" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="B222" s="2" t="n">
         <v>54310.694334358</v>
@@ -15561,7 +15571,7 @@
     </row>
     <row r="223">
       <c r="A223" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B223" s="2" t="n">
         <v>49169.3526191725</v>
@@ -15620,7 +15630,7 @@
     </row>
     <row r="224">
       <c r="A224" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="B224" s="2" t="n">
         <v>50983.5724258489</v>
@@ -15679,7 +15689,7 @@
     </row>
     <row r="225">
       <c r="A225" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B225" s="2" t="n">
         <v>48857.4806586734</v>
@@ -15738,7 +15748,7 @@
     </row>
     <row r="226">
       <c r="A226" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B226" s="2" t="n">
         <v>48753.9260014278</v>
@@ -15797,7 +15807,7 @@
     </row>
     <row r="227">
       <c r="A227" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B227" s="2" t="n">
         <v>51364.2942847664</v>
@@ -15856,7 +15866,7 @@
     </row>
     <row r="228">
       <c r="A228" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B228" s="2" t="n">
         <v>48873.5995738463</v>
@@ -15915,7 +15925,7 @@
     </row>
     <row r="229">
       <c r="A229" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B229" s="2" t="n">
         <v>46657.0586072988</v>
@@ -15974,7 +15984,7 @@
     </row>
     <row r="230">
       <c r="A230" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B230" s="2" t="n">
         <v>51756.106246975</v>
@@ -16033,7 +16043,7 @@
     </row>
     <row r="231">
       <c r="A231" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B231" s="2" t="n">
         <v>46377.077710561</v>
@@ -16092,7 +16102,7 @@
     </row>
     <row r="232">
       <c r="A232" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="B232" s="2" t="n">
         <v>53109.0594080509</v>
@@ -16151,7 +16161,7 @@
     </row>
     <row r="233">
       <c r="A233" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B233" s="2" t="n">
         <v>56708.0390184044</v>
@@ -16210,7 +16220,7 @@
     </row>
     <row r="234">
       <c r="A234" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="B234" s="2" t="n">
         <v>59507.7841626455</v>
@@ -16269,7 +16279,7 @@
     </row>
     <row r="235">
       <c r="A235" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="B235" s="2" t="n">
         <v>52930.8490880637</v>
@@ -16328,7 +16338,7 @@
     </row>
     <row r="236">
       <c r="A236" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B236" s="2" t="n">
         <v>62432.9691879827</v>
@@ -16387,7 +16397,7 @@
     </row>
     <row r="237">
       <c r="A237" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B237" s="2" t="n">
         <v>57767.0613852806</v>
@@ -16446,7 +16456,7 @@
     </row>
     <row r="238">
       <c r="A238" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="B238" s="2" t="n">
         <v>57628.1938696784</v>
@@ -16505,7 +16515,7 @@
     </row>
     <row r="239">
       <c r="A239" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B239" s="2" t="n">
         <v>57670.0296057783</v>
@@ -16564,7 +16574,7 @@
     </row>
     <row r="240">
       <c r="A240" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="B240" s="2" t="n">
         <v>52140.4887568409</v>
@@ -16623,7 +16633,7 @@
     </row>
     <row r="241">
       <c r="A241" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B241" s="2" t="n">
         <v>52708.6014773433</v>
@@ -16682,7 +16692,7 @@
     </row>
     <row r="242">
       <c r="A242" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="B242" s="2" t="n">
         <v>53061.2584519036</v>
@@ -16741,7 +16751,7 @@
     </row>
     <row r="243">
       <c r="A243" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B243" s="2" t="n">
         <v>47053.1655514512</v>
@@ -16800,7 +16810,7 @@
     </row>
     <row r="244">
       <c r="A244" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B244" s="2" t="n">
         <v>53577.7894997067</v>
@@ -16859,7 +16869,7 @@
     </row>
     <row r="245">
       <c r="A245" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B245" s="2" t="n">
         <v>53496.735079329</v>
@@ -16918,7 +16928,7 @@
     </row>
     <row r="246">
       <c r="A246" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B246" s="2" t="n">
         <v>56491.306017889</v>
@@ -16977,7 +16987,7 @@
     </row>
     <row r="247">
       <c r="A247" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B247" s="2" t="n">
         <v>56854.8760860058</v>
@@ -17036,7 +17046,7 @@
     </row>
     <row r="248">
       <c r="A248" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="B248" s="2" t="n">
         <v>56155.456409365</v>
@@ -17095,7 +17105,7 @@
     </row>
     <row r="249">
       <c r="A249" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B249" s="2" t="n">
         <v>53338.172509239</v>
@@ -17154,7 +17164,7 @@
     </row>
     <row r="250">
       <c r="A250" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="B250" s="2" t="n">
         <v>57365.8625323501</v>
@@ -17213,7 +17223,7 @@
     </row>
     <row r="251">
       <c r="A251" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B251" s="2" t="n">
         <v>56866.4969690701</v>
@@ -17272,7 +17282,7 @@
     </row>
     <row r="252">
       <c r="A252" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B252" s="2" t="n">
         <v>48925.5803305003</v>
@@ -17331,7 +17341,7 @@
     </row>
     <row r="253">
       <c r="A253" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B253" s="2" t="n">
         <v>52131.911084876</v>
@@ -17390,7 +17400,7 @@
     </row>
     <row r="254">
       <c r="A254" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B254" s="2" t="n">
         <v>61376.2365070231</v>
@@ -17449,7 +17459,7 @@
     </row>
     <row r="255">
       <c r="A255" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B255" s="2" t="n">
         <v>54756.5906457855</v>
@@ -17508,7 +17518,7 @@
     </row>
     <row r="256">
       <c r="A256" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="B256" s="2" t="n">
         <v>60608.4829099297</v>
@@ -17567,7 +17577,7 @@
     </row>
     <row r="257">
       <c r="A257" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B257" s="2" t="n">
         <v>59770.0249014401</v>
@@ -17626,7 +17636,7 @@
     </row>
     <row r="258">
       <c r="A258" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B258" s="2" t="n">
         <v>57073.9823653985</v>
@@ -17685,7 +17695,7 @@
     </row>
     <row r="259">
       <c r="A259" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B259" s="2" t="n">
         <v>64019.0213056353</v>
@@ -17744,7 +17754,7 @@
     </row>
     <row r="260">
       <c r="A260" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="B260" s="2" t="n">
         <v>58842.5697031276</v>
@@ -17803,7 +17813,7 @@
     </row>
     <row r="261">
       <c r="A261" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B261" s="2" t="n">
         <v>55190.2473327112</v>
@@ -17862,7 +17872,7 @@
     </row>
     <row r="262">
       <c r="A262" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="B262" s="2" t="n">
         <v>56618.5281014779</v>
@@ -17921,7 +17931,7 @@
     </row>
     <row r="263">
       <c r="A263" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B263" s="2" t="n">
         <v>54288.1302254726</v>
@@ -17980,7 +17990,7 @@
     </row>
     <row r="264">
       <c r="A264" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B264" s="2" t="n">
         <v>49885.3208160131</v>
@@ -18039,7 +18049,7 @@
     </row>
     <row r="265">
       <c r="A265" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="B265" s="2" t="n">
         <v>49464.1641379116</v>
@@ -18098,7 +18108,7 @@
     </row>
     <row r="266">
       <c r="A266" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B266" s="2" t="n">
         <v>51438.6328636363</v>
@@ -18157,7 +18167,7 @@
     </row>
     <row r="267">
       <c r="A267" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="B267" s="2" t="n">
         <v>49512.2335023431</v>
@@ -18216,7 +18226,7 @@
     </row>
     <row r="268">
       <c r="A268" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B268" s="2" t="n">
         <v>57225.555355058</v>
@@ -18275,7 +18285,7 @@
     </row>
     <row r="269">
       <c r="A269" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="B269" s="2" t="n">
         <v>48935.7040898593</v>
@@ -18334,7 +18344,7 @@
     </row>
     <row r="270">
       <c r="A270" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B270" s="2" t="n">
         <v>56476.3908840634</v>
@@ -18393,7 +18403,7 @@
     </row>
     <row r="271">
       <c r="A271" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B271" s="2" t="n">
         <v>51945.0717714809</v>
@@ -18452,7 +18462,7 @@
     </row>
     <row r="272">
       <c r="A272" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B272" s="2" t="n">
         <v>52188.6562189585</v>
@@ -18511,7 +18521,7 @@
     </row>
     <row r="273">
       <c r="A273" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="B273" s="2" t="n">
         <v>58529.9452800634</v>
@@ -18570,7 +18580,7 @@
     </row>
     <row r="274">
       <c r="A274" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B274" s="2" t="n">
         <v>53836.517657819</v>
@@ -18629,7 +18639,7 @@
     </row>
     <row r="275">
       <c r="A275" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B275" s="2" t="n">
         <v>48516.9846139502</v>
@@ -18688,7 +18698,7 @@
     </row>
     <row r="276">
       <c r="A276" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B276" s="2" t="n">
         <v>53978.8564522728</v>
@@ -18747,7 +18757,7 @@
     </row>
     <row r="277">
       <c r="A277" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B277" s="2" t="n">
         <v>54083.7780213846</v>
@@ -18806,7 +18816,7 @@
     </row>
     <row r="278">
       <c r="A278" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B278" s="2" t="n">
         <v>54863.7918488072</v>
@@ -18865,7 +18875,7 @@
     </row>
     <row r="279">
       <c r="A279" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B279" s="2" t="n">
         <v>47403.2124084582</v>
@@ -18924,7 +18934,7 @@
     </row>
     <row r="280">
       <c r="A280" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B280" s="2" t="n">
         <v>59049.5283460073</v>
@@ -18983,7 +18993,7 @@
     </row>
     <row r="281">
       <c r="A281" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="B281" s="2" t="n">
         <v>49136.8803462985</v>
@@ -19042,7 +19052,7 @@
     </row>
     <row r="282">
       <c r="A282" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B282" s="2" t="n">
         <v>58644.3672212872</v>
@@ -19101,7 +19111,7 @@
     </row>
     <row r="283">
       <c r="A283" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B283" s="2" t="n">
         <v>57807.3753913517</v>
@@ -19160,7 +19170,7 @@
     </row>
     <row r="284">
       <c r="A284" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B284" s="2" t="n">
         <v>54824.6607718645</v>
@@ -19219,7 +19229,7 @@
     </row>
     <row r="285">
       <c r="A285" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B285" s="2" t="n">
         <v>58172.0284746239</v>
@@ -19278,7 +19288,7 @@
     </row>
     <row r="286">
       <c r="A286" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="B286" s="2" t="n">
         <v>56581.689824747</v>
@@ -19337,7 +19347,7 @@
     </row>
     <row r="287">
       <c r="A287" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B287" s="2" t="n">
         <v>59662.2564373069</v>
@@ -19396,7 +19406,7 @@
     </row>
     <row r="288">
       <c r="A288" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="B288" s="2" t="n">
         <v>58894.0734979197</v>
@@ -19455,7 +19465,7 @@
     </row>
     <row r="289">
       <c r="A289" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="B289" s="2" t="n">
         <v>55368.5668756009</v>
@@ -19514,7 +19524,7 @@
     </row>
     <row r="290">
       <c r="A290" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B290" s="2" t="n">
         <v>60962.2203057882</v>
@@ -19573,7 +19583,7 @@
     </row>
     <row r="291">
       <c r="A291" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="B291" s="2" t="n">
         <v>54175.4972513408</v>
@@ -19632,7 +19642,7 @@
     </row>
     <row r="292">
       <c r="A292" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B292" s="2" t="n">
         <v>63466.7259151895</v>
@@ -19691,7 +19701,7 @@
     </row>
     <row r="293">
       <c r="A293" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="B293" s="2" t="n">
         <v>59411.0426048424</v>
@@ -19750,7 +19760,7 @@
     </row>
     <row r="294">
       <c r="A294" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B294" s="2" t="n">
         <v>62057.8496285042</v>
@@ -19809,7 +19819,7 @@
     </row>
     <row r="295">
       <c r="A295" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B295" s="2" t="n">
         <v>59531.0485588665</v>
@@ -19868,7 +19878,7 @@
     </row>
     <row r="296">
       <c r="A296" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B296" s="2" t="n">
         <v>64963.440314047</v>
@@ -19927,7 +19937,7 @@
     </row>
     <row r="297">
       <c r="A297" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="B297" s="2" t="n">
         <v>65796.084170749</v>
@@ -19986,7 +19996,7 @@
     </row>
     <row r="298">
       <c r="A298" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B298" s="2" t="n">
         <v>57406.5707736888</v>
@@ -20045,7 +20055,7 @@
     </row>
     <row r="299">
       <c r="A299" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B299" s="2" t="n">
         <v>67099.4248158723</v>
@@ -20104,7 +20114,7 @@
     </row>
     <row r="300">
       <c r="A300" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B300" s="2" t="n">
         <v>62873.2105604545</v>
@@ -20163,7 +20173,7 @@
     </row>
     <row r="301">
       <c r="A301" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="B301" s="2" t="n">
         <v>59477.6938174954</v>
@@ -20222,7 +20232,7 @@
     </row>
     <row r="302">
       <c r="A302" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B302" s="2" t="n">
         <v>63871.0876333924</v>
@@ -20281,7 +20291,7 @@
     </row>
     <row r="303">
       <c r="A303" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="B303" s="2" t="n">
         <v>56190.0568719834</v>
@@ -20340,7 +20350,7 @@
     </row>
     <row r="304">
       <c r="A304" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B304" s="2" t="n">
         <v>58306.3476154771</v>
@@ -20399,7 +20409,7 @@
     </row>
     <row r="305">
       <c r="A305" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B305" s="2" t="n">
         <v>61247.0802329513</v>
@@ -20458,7 +20468,7 @@
     </row>
     <row r="306">
       <c r="A306" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B306" s="2" t="n">
         <v>66799.6866716514</v>
@@ -20517,7 +20527,7 @@
     </row>
     <row r="307">
       <c r="A307" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B307" s="2" t="n">
         <v>59576.1782368075</v>
@@ -20576,7 +20586,7 @@
     </row>
     <row r="308">
       <c r="A308" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B308" s="2" t="n">
         <v>70169.1655170679</v>
@@ -20635,7 +20645,7 @@
     </row>
     <row r="309">
       <c r="A309" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="B309" s="2" t="n">
         <v>66499.5391451826</v>
@@ -20694,7 +20704,7 @@
     </row>
     <row r="310">
       <c r="A310" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B310" s="2" t="n">
         <v>67667.2591680449</v>
@@ -20753,7 +20763,7 @@
     </row>
     <row r="311">
       <c r="A311" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B311" s="2" t="n">
         <v>75060.0618879841</v>
@@ -20812,7 +20822,7 @@
     </row>
     <row r="312">
       <c r="A312" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B312" s="2" t="n">
         <v>67024.7794861448</v>
@@ -20871,7 +20881,7 @@
     </row>
     <row r="313">
       <c r="A313" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="B313" s="2" t="n">
         <v>67659.6225102471</v>
@@ -20930,7 +20940,7 @@
     </row>
     <row r="314">
       <c r="A314" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B314" s="2" t="n">
         <v>63693.7045254554</v>
@@ -20989,7 +20999,7 @@
     </row>
     <row r="315">
       <c r="A315" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="B315" s="2" t="n">
         <v>53612.8983171627</v>
@@ -21048,7 +21058,7 @@
     </row>
     <row r="316">
       <c r="A316" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B316" s="2" t="n">
         <v>59420.2246878659</v>
@@ -21107,7 +21117,7 @@
     </row>
     <row r="317">
       <c r="A317" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B317" s="2" t="n">
         <v>66346.5882334129</v>
@@ -21166,7 +21176,7 @@
     </row>
     <row r="318">
       <c r="A318" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="B318" s="2" t="n">
         <v>63280.6812266243</v>
@@ -21225,7 +21235,7 @@
     </row>
     <row r="319">
       <c r="A319" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B319" s="2" t="n">
         <v>68264.594717033</v>
@@ -21284,7 +21294,7 @@
     </row>
     <row r="320">
       <c r="A320" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="B320" s="2" t="n">
         <v>72508.5716165972</v>
@@ -21343,7 +21353,7 @@
     </row>
     <row r="321">
       <c r="A321" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B321" s="2" t="n">
         <v>66750.1255689499</v>
@@ -21402,7 +21412,7 @@
     </row>
     <row r="322">
       <c r="A322" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="B322" s="2" t="n">
         <v>64111.4715276129</v>
@@ -21461,7 +21471,7 @@
     </row>
     <row r="323">
       <c r="A323" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B323" s="2" t="n">
         <v>67673.2264346566</v>
@@ -21520,7 +21530,7 @@
     </row>
     <row r="324">
       <c r="A324" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B324" s="2" t="n">
         <v>65828.5828409713</v>
@@ -21579,7 +21589,7 @@
     </row>
     <row r="325">
       <c r="A325" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B325" s="2" t="n">
         <v>61770.96837903</v>
@@ -21638,7 +21648,7 @@
     </row>
     <row r="326">
       <c r="A326" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="B326" s="2" t="n">
         <v>57065.4058718966</v>
@@ -21697,7 +21707,7 @@
     </row>
     <row r="327">
       <c r="A327" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B327" s="2" t="n">
         <v>55275.6518289698</v>
@@ -21756,7 +21766,7 @@
     </row>
     <row r="328">
       <c r="A328" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="B328" s="2" t="n">
         <v>68216.0181964318</v>
@@ -21815,7 +21825,7 @@
     </row>
     <row r="329">
       <c r="A329" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B329" s="2" t="n">
         <v>63462.0106096671</v>
@@ -21874,7 +21884,7 @@
     </row>
     <row r="330">
       <c r="A330" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="B330" s="2" t="n">
         <v>56300.7739366472</v>
@@ -21933,7 +21943,7 @@
     </row>
     <row r="331">
       <c r="A331" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B331" s="2" t="n">
         <v>63527.5087758916</v>
@@ -21992,7 +22002,7 @@
     </row>
     <row r="332">
       <c r="A332" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="B332" s="2" t="n">
         <v>66396.5962512514</v>
@@ -22051,7 +22061,7 @@
     </row>
     <row r="333">
       <c r="A333" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B333" s="2" t="n">
         <v>68222.4053055153</v>
@@ -22110,7 +22120,7 @@
     </row>
     <row r="334">
       <c r="A334" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="B334" s="2" t="n">
         <v>65613.5433526452</v>
@@ -22169,7 +22179,7 @@
     </row>
     <row r="335">
       <c r="A335" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="B335" s="2" t="n">
         <v>62352.954846695</v>
@@ -22228,7 +22238,7 @@
     </row>
     <row r="336">
       <c r="A336" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B336" s="2" t="n">
         <v>63373.2860268065</v>
@@ -22287,7 +22297,7 @@
     </row>
     <row r="337">
       <c r="A337" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B337" s="2" t="n">
         <v>66396.4268140794</v>
@@ -22346,7 +22356,7 @@
     </row>
     <row r="338">
       <c r="A338" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="B338" s="2" t="n">
         <v>54836.6052750205</v>
@@ -22405,7 +22415,7 @@
     </row>
     <row r="339">
       <c r="A339" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="B339" s="2" t="n">
         <v>59163.3898832853</v>
@@ -22464,7 +22474,7 @@
     </row>
     <row r="340">
       <c r="A340" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B340" s="2" t="n">
         <v>67291.3991368405</v>
@@ -22523,7 +22533,7 @@
     </row>
     <row r="341">
       <c r="A341" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B341" s="2" t="n">
         <v>61857.6265767347</v>
@@ -22582,7 +22592,7 @@
     </row>
     <row r="342">
       <c r="A342" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B342" s="2" t="n">
         <v>68701.871189</v>
@@ -22641,7 +22651,7 @@
     </row>
     <row r="343">
       <c r="A343" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="B343" s="2" t="n">
         <v>67924.6244782047</v>
@@ -22700,7 +22710,7 @@
     </row>
     <row r="344">
       <c r="A344" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B344" s="2" t="n">
         <v>69619.3417574073</v>
@@ -22759,7 +22769,7 @@
     </row>
     <row r="345">
       <c r="A345" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="B345" s="2" t="n">
         <v>72189.9752840389</v>
@@ -22818,7 +22828,7 @@
     </row>
     <row r="346">
       <c r="A346" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B346" s="2" t="n">
         <v>69400.6837348512</v>
@@ -22877,7 +22887,7 @@
     </row>
     <row r="347">
       <c r="A347" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B347" s="2" t="n">
         <v>60450.387591882</v>
@@ -22936,7 +22946,7 @@
     </row>
     <row r="348">
       <c r="A348" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B348" s="2" t="n">
         <v>65767.4048478929</v>
@@ -22995,7 +23005,7 @@
     </row>
     <row r="349">
       <c r="A349" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B349" s="2" t="n">
         <v>66299.6788838283</v>
@@ -23054,7 +23064,7 @@
     </row>
     <row r="350">
       <c r="A350" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B350" s="2" t="n">
         <v>66708.3251570389</v>
@@ -23113,7 +23123,7 @@
     </row>
     <row r="351">
       <c r="A351" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="B351" s="2" t="n">
         <v>57584.7539989328</v>
@@ -23172,7 +23182,7 @@
     </row>
     <row r="352">
       <c r="A352" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B352" s="2" t="n">
         <v>71170.6964138567</v>
@@ -23231,7 +23241,7 @@
     </row>
     <row r="353">
       <c r="A353" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="B353" s="2" t="n">
         <v>62861.3574675856</v>
@@ -23290,7 +23300,7 @@
     </row>
     <row r="354">
       <c r="A354" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="B354" s="2" t="n">
         <v>69705.4334805234</v>
@@ -23349,7 +23359,7 @@
     </row>
     <row r="355">
       <c r="A355" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B355" s="2" t="n">
         <v>70998.990048854</v>
@@ -23408,7 +23418,7 @@
     </row>
     <row r="356">
       <c r="A356" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B356" s="2" t="n">
         <v>71003.5215918672</v>
@@ -23467,7 +23477,7 @@
     </row>
     <row r="357">
       <c r="A357" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B357" s="2" t="n">
         <v>67025.9371578543</v>
@@ -23526,7 +23536,7 @@
     </row>
     <row r="358">
       <c r="A358" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B358" s="2" t="n">
         <v>65071.1272557081</v>
@@ -23585,7 +23595,7 @@
     </row>
     <row r="359">
       <c r="A359" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B359" s="2" t="n">
         <v>60779.4274515912</v>
@@ -23644,7 +23654,7 @@
     </row>
     <row r="360">
       <c r="A360" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="B360" s="2" t="n">
         <v>67980.8162776186</v>
@@ -23703,7 +23713,7 @@
     </row>
     <row r="361">
       <c r="A361" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B361" s="2" t="n">
         <v>60677.7320456823</v>
@@ -23762,7 +23772,7 @@
     </row>
     <row r="362">
       <c r="A362" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B362" s="2" t="n">
         <v>69941.0354357389</v>
@@ -23821,7 +23831,7 @@
     </row>
     <row r="363">
       <c r="A363" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B363" s="2" t="n">
         <v>60209.3743811086</v>
@@ -23880,7 +23890,7 @@
     </row>
     <row r="364">
       <c r="A364" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B364" s="2" t="n">
         <v>61431.2388742256</v>
@@ -23939,7 +23949,7 @@
     </row>
     <row r="365">
       <c r="A365" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B365" s="2" t="n">
         <v>60280.6465115254</v>
@@ -23998,7 +24008,7 @@
     </row>
     <row r="366">
       <c r="A366" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B366" s="2" t="n">
         <v>67567.3299667724</v>
@@ -24057,7 +24067,7 @@
     </row>
     <row r="367">
       <c r="A367" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B367" s="2" t="n">
         <v>60424.8747986739</v>
@@ -24116,7 +24126,7 @@
     </row>
     <row r="368">
       <c r="A368" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="B368" s="2" t="n">
         <v>74921.7008102218</v>
@@ -24175,7 +24185,7 @@
     </row>
     <row r="369">
       <c r="A369" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B369" s="2" t="n">
         <v>69802.282062254</v>
@@ -24234,7 +24244,7 @@
     </row>
     <row r="370">
       <c r="A370" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="B370" s="2" t="n">
         <v>66588.9606911919</v>
@@ -24293,7 +24303,7 @@
     </row>
     <row r="371">
       <c r="A371" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="B371" s="2" t="n">
         <v>68935.7248077474</v>
@@ -24352,7 +24362,7 @@
     </row>
     <row r="372">
       <c r="A372" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B372" s="2" t="n">
         <v>62853.4586430954</v>
@@ -24411,7 +24421,7 @@
     </row>
     <row r="373">
       <c r="A373" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B373" s="2" t="n">
         <v>69913.3770075089</v>
@@ -24470,7 +24480,7 @@
     </row>
     <row r="374">
       <c r="A374" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B374" s="2" t="n">
         <v>67519.2553963051</v>
@@ -24529,7 +24539,7 @@
     </row>
     <row r="375">
       <c r="A375" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B375" s="2" t="n">
         <v>59233.4711957493</v>
@@ -24588,7 +24598,7 @@
     </row>
     <row r="376">
       <c r="A376" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B376" s="2" t="n">
         <v>60254.5972537374</v>
@@ -24647,7 +24657,7 @@
     </row>
     <row r="377">
       <c r="A377" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B377" s="2" t="n">
         <v>66244.4306040227</v>
@@ -24706,7 +24716,7 @@
     </row>
     <row r="378">
       <c r="A378" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B378" s="2" t="n">
         <v>70143.6678297847</v>
@@ -24765,7 +24775,7 @@
     </row>
     <row r="379">
       <c r="A379" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="B379" s="2" t="n">
         <v>67220.6316272751</v>
@@ -24824,7 +24834,7 @@
     </row>
     <row r="380">
       <c r="A380" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="B380" s="2" t="n">
         <v>75558.7961711049</v>
@@ -24883,7 +24893,7 @@
     </row>
     <row r="381">
       <c r="A381" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B381" s="2" t="n">
         <v>71033.7965845084</v>
@@ -24942,7 +24952,7 @@
     </row>
     <row r="382">
       <c r="A382" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B382" s="2" t="n">
         <v>69627.7223841994</v>
@@ -25001,7 +25011,7 @@
     </row>
     <row r="383">
       <c r="A383" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B383" s="2" t="n">
         <v>70966.8415899281</v>
@@ -25060,7 +25070,7 @@
     </row>
     <row r="384">
       <c r="A384" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B384" s="2" t="n">
         <v>64902.0507950805</v>
@@ -25119,7 +25129,7 @@
     </row>
     <row r="385">
       <c r="A385" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B385" s="2" t="n">
         <v>70382.46269184</v>
@@ -25178,7 +25188,7 @@
     </row>
     <row r="386">
       <c r="A386" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="B386" s="2" t="n">
         <v>66093.0743226928</v>
@@ -25237,7 +25247,7 @@
     </row>
     <row r="387">
       <c r="A387" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B387" s="2" t="n">
         <v>59243.298900064</v>
@@ -25296,7 +25306,7 @@
     </row>
     <row r="388">
       <c r="A388" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="B388" s="2" t="n">
         <v>69361.5470713869</v>
@@ -25355,7 +25365,7 @@
     </row>
     <row r="389">
       <c r="A389" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B389" s="2" t="n">
         <v>63190.83882223</v>
@@ -25414,7 +25424,7 @@
     </row>
     <row r="390">
       <c r="A390" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="B390" s="2"/>
       <c r="C390" s="3" t="n">
@@ -25445,7 +25455,7 @@
     </row>
     <row r="391">
       <c r="A391" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B391" s="2"/>
       <c r="C391" s="3" t="n">
@@ -25476,7 +25486,7 @@
     </row>
     <row r="392">
       <c r="A392" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B392" s="2"/>
       <c r="C392" s="3" t="n">
@@ -25507,7 +25517,7 @@
     </row>
     <row r="393">
       <c r="A393" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B393" s="2"/>
       <c r="C393" s="3" t="n">
@@ -25538,7 +25548,7 @@
     </row>
     <row r="394">
       <c r="A394" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="B394" s="2"/>
       <c r="C394" s="3" t="n">
@@ -25569,7 +25579,7 @@
     </row>
     <row r="395">
       <c r="A395" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B395" s="2"/>
       <c r="C395" s="3" t="n">
@@ -25600,7 +25610,7 @@
     </row>
     <row r="396">
       <c r="A396" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="B396" s="2"/>
       <c r="C396" s="3" t="n">
@@ -25631,7 +25641,7 @@
     </row>
     <row r="397">
       <c r="A397" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B397" s="2"/>
       <c r="C397" s="3" t="n">
@@ -25662,7 +25672,7 @@
     </row>
     <row r="398">
       <c r="A398" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B398" s="2"/>
       <c r="C398" s="3" t="n">
@@ -25693,7 +25703,7 @@
     </row>
     <row r="399">
       <c r="A399" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="B399" s="2"/>
       <c r="C399" s="3" t="n">
@@ -25724,7 +25734,7 @@
     </row>
     <row r="400">
       <c r="A400" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B400" s="2"/>
       <c r="C400" s="3" t="n">
@@ -25755,7 +25765,7 @@
     </row>
     <row r="401">
       <c r="A401" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="B401" s="2"/>
       <c r="C401" s="3" t="n">
@@ -25786,7 +25796,7 @@
     </row>
     <row r="402">
       <c r="A402" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B402" s="2"/>
       <c r="C402" s="3"/>
@@ -25809,7 +25819,7 @@
     </row>
     <row r="403">
       <c r="A403" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B403" s="2"/>
       <c r="C403" s="3"/>
@@ -25832,7 +25842,7 @@
     </row>
     <row r="404">
       <c r="A404" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B404" s="2"/>
       <c r="C404" s="3"/>
@@ -25855,7 +25865,7 @@
     </row>
     <row r="405">
       <c r="A405" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="B405" s="2"/>
       <c r="C405" s="3"/>
@@ -25878,7 +25888,7 @@
     </row>
     <row r="406">
       <c r="A406" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B406" s="2"/>
       <c r="C406" s="3"/>
@@ -25901,7 +25911,7 @@
     </row>
     <row r="407">
       <c r="A407" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="B407" s="2"/>
       <c r="C407" s="3"/>
@@ -25924,7 +25934,7 @@
     </row>
     <row r="408">
       <c r="A408" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="B408" s="2"/>
       <c r="C408" s="3"/>
@@ -25947,7 +25957,7 @@
     </row>
     <row r="409">
       <c r="A409" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B409" s="2"/>
       <c r="C409" s="3"/>
@@ -25970,7 +25980,7 @@
     </row>
     <row r="410">
       <c r="A410" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="B410" s="2"/>
       <c r="C410" s="3"/>
@@ -25993,7 +26003,7 @@
     </row>
     <row r="411">
       <c r="A411" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="B411" s="2"/>
       <c r="C411" s="3"/>
@@ -26016,7 +26026,7 @@
     </row>
     <row r="412">
       <c r="A412" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="B412" s="2"/>
       <c r="C412" s="3"/>
@@ -26039,7 +26049,7 @@
     </row>
     <row r="413">
       <c r="A413" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B413" s="2"/>
       <c r="C413" s="3"/>
@@ -26062,7 +26072,7 @@
     </row>
     <row r="414">
       <c r="A414" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="B414" s="2"/>
       <c r="C414" s="3"/>
@@ -26085,7 +26095,7 @@
     </row>
     <row r="415">
       <c r="A415" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B415" s="2"/>
       <c r="C415" s="3"/>
@@ -26108,7 +26118,7 @@
     </row>
     <row r="416">
       <c r="A416" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B416" s="2"/>
       <c r="C416" s="3"/>
@@ -26131,7 +26141,7 @@
     </row>
     <row r="417">
       <c r="A417" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B417" s="2"/>
       <c r="C417" s="3"/>
@@ -26154,7 +26164,7 @@
     </row>
     <row r="418">
       <c r="A418" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B418" s="2"/>
       <c r="C418" s="3"/>
@@ -26177,7 +26187,7 @@
     </row>
     <row r="419">
       <c r="A419" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="B419" s="2"/>
       <c r="C419" s="3"/>
@@ -26200,7 +26210,7 @@
     </row>
     <row r="420">
       <c r="A420" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B420" s="2"/>
       <c r="C420" s="3"/>
@@ -26223,7 +26233,7 @@
     </row>
     <row r="421">
       <c r="A421" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="B421" s="2"/>
       <c r="C421" s="3"/>
@@ -26246,7 +26256,7 @@
     </row>
     <row r="422">
       <c r="A422" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="B422" s="2"/>
       <c r="C422" s="3"/>
@@ -26269,7 +26279,7 @@
     </row>
     <row r="423">
       <c r="A423" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B423" s="2"/>
       <c r="C423" s="3"/>
@@ -26292,7 +26302,7 @@
     </row>
     <row r="424">
       <c r="A424" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="B424" s="2"/>
       <c r="C424" s="3"/>
@@ -26315,7 +26325,7 @@
     </row>
     <row r="425">
       <c r="A425" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B425" s="2"/>
       <c r="C425" s="3"/>
@@ -26338,7 +26348,7 @@
     </row>
     <row r="426">
       <c r="A426" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="B426" s="2"/>
       <c r="C426" s="3"/>
@@ -26361,7 +26371,7 @@
     </row>
     <row r="427">
       <c r="A427" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B427" s="2"/>
       <c r="C427" s="3"/>
@@ -26384,7 +26394,7 @@
     </row>
     <row r="428">
       <c r="A428" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="B428" s="2"/>
       <c r="C428" s="3"/>
@@ -26407,7 +26417,7 @@
     </row>
     <row r="429">
       <c r="A429" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B429" s="2"/>
       <c r="C429" s="3"/>
@@ -26430,7 +26440,7 @@
     </row>
     <row r="430">
       <c r="A430" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="B430" s="2"/>
       <c r="C430" s="3"/>
@@ -26453,7 +26463,7 @@
     </row>
     <row r="431">
       <c r="A431" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B431" s="2"/>
       <c r="C431" s="3"/>
@@ -26476,7 +26486,7 @@
     </row>
     <row r="432">
       <c r="A432" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="B432" s="2"/>
       <c r="C432" s="3"/>
@@ -26499,7 +26509,7 @@
     </row>
     <row r="433">
       <c r="A433" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B433" s="2"/>
       <c r="C433" s="3"/>
@@ -26522,7 +26532,7 @@
     </row>
     <row r="434">
       <c r="A434" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B434" s="2"/>
       <c r="C434" s="3"/>
@@ -26545,7 +26555,7 @@
     </row>
     <row r="435">
       <c r="A435" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="B435" s="2"/>
       <c r="C435" s="3"/>
@@ -26568,7 +26578,7 @@
     </row>
     <row r="436">
       <c r="A436" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B436" s="2"/>
       <c r="C436" s="3"/>
@@ -26591,7 +26601,7 @@
     </row>
     <row r="437">
       <c r="A437" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="B437" s="2"/>
       <c r="C437" s="3"/>
@@ -26614,7 +26624,7 @@
     </row>
     <row r="438">
       <c r="A438" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B438" s="2"/>
       <c r="C438" s="3"/>
@@ -26637,7 +26647,7 @@
     </row>
     <row r="439">
       <c r="A439" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B439" s="2"/>
       <c r="C439" s="3"/>
@@ -26660,7 +26670,7 @@
     </row>
     <row r="440">
       <c r="A440" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B440" s="2"/>
       <c r="C440" s="3"/>
@@ -26683,7 +26693,7 @@
     </row>
     <row r="441">
       <c r="A441" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="B441" s="2"/>
       <c r="C441" s="3"/>
@@ -26706,7 +26716,7 @@
     </row>
     <row r="442">
       <c r="A442" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B442" s="2"/>
       <c r="C442" s="3"/>
@@ -26729,7 +26739,7 @@
     </row>
     <row r="443">
       <c r="A443" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B443" s="2"/>
       <c r="C443" s="3"/>
@@ -26752,7 +26762,7 @@
     </row>
     <row r="444">
       <c r="A444" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="B444" s="2"/>
       <c r="C444" s="3"/>
@@ -26775,7 +26785,7 @@
     </row>
     <row r="445">
       <c r="A445" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="B445" s="2"/>
       <c r="C445" s="3"/>
@@ -26809,97 +26819,97 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
     </row>
   </sheetData>
@@ -26923,7 +26933,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -26933,13 +26943,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>-0.0282381544450935</v>
@@ -26947,7 +26957,7 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>-0.00563100374805844</v>
@@ -26955,7 +26965,7 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>-0.0011446585140367</v>
@@ -26963,7 +26973,7 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>0.00192534427605877</v>
@@ -26971,7 +26981,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B9" s="1" t="n">
         <v>-0.00356754737306025</v>
@@ -26979,7 +26989,7 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>-0.0384770885629665</v>
@@ -26987,7 +26997,7 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>-0.0735579310077793</v>
@@ -26995,7 +27005,7 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B12" s="1" t="n">
         <v>-0.0436931966897479</v>
@@ -27003,7 +27013,7 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>0.0313928970039379</v>
@@ -27011,7 +27021,7 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="B14" s="1" t="n">
         <v>0.0666854335944708</v>
@@ -27019,7 +27029,7 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B15" s="1" t="n">
         <v>0.0290725174781228</v>
@@ -27027,7 +27037,7 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B16" s="1" t="n">
         <v>-0.00911985480690611</v>
@@ -27035,7 +27045,7 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B17" s="1" t="n">
         <v>-0.0276190566992275</v>
@@ -27043,7 +27053,7 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>-0.0385299441523951</v>
@@ -27051,7 +27061,7 @@
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="B19" s="1" t="n">
         <v>-0.00646123107566736</v>
@@ -27059,7 +27069,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B20" s="1" t="n">
         <v>0.0205583850470838</v>
@@ -27067,7 +27077,7 @@
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B21" s="1" t="n">
         <v>0.00976651431134003</v>
@@ -27075,7 +27085,7 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>0.0258907283291465</v>
@@ -27083,7 +27093,7 @@
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="B23" s="1" t="n">
         <v>0.0733839550141418</v>

</xml_diff>

<commit_message>
Corrida | SFE-FAEN | 2026-08-14 10:05:16.008186
</commit_message>
<xml_diff>
--- a/indicadores/SFE-FAEN_out.xlsx
+++ b/indicadores/SFE-FAEN_out.xlsx
@@ -104,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">13/07/2026</t>
+    <t xml:space="preserve">14/08/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">fleiva</t>
+    <t xml:space="preserve">arodriguez</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -2181,7 +2181,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>-0.0732862388760376</v>
+        <v>0.0601505331301639</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -2197,7 +2197,7 @@
       <c r="B12"/>
       <c r="C12"/>
       <c r="D12" t="n">
-        <v>-3</v>
+        <v>9</v>
       </c>
       <c r="E12"/>
       <c r="F12"/>
@@ -2239,7 +2239,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.00457335517530832</v>
+        <v>0.00328515173732875</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -2309,7 +2309,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.194826459504615</v>
+        <v>0.253113330624314</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2339,7 +2339,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.916646126240233</v>
+        <v>0.958514814762758</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -26988,7 +26988,7 @@
         <v>516</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0283859861275433</v>
+        <v>-0.0378983610678733</v>
       </c>
     </row>
     <row r="6">
@@ -26996,7 +26996,7 @@
         <v>517</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.00696357591621302</v>
+        <v>-0.0167124012997013</v>
       </c>
     </row>
     <row r="7">
@@ -27004,7 +27004,7 @@
         <v>518</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>0.00167656922012304</v>
+        <v>-0.00230447995817254</v>
       </c>
     </row>
     <row r="8">
@@ -27012,7 +27012,7 @@
         <v>519</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.00429067374022802</v>
+        <v>-0.00318693624772995</v>
       </c>
     </row>
     <row r="9">
@@ -27020,7 +27020,7 @@
         <v>520</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>-0.00635337980064308</v>
+        <v>-0.0168985050001984</v>
       </c>
     </row>
     <row r="10">
@@ -27028,7 +27028,7 @@
         <v>521</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>-0.0462787649256719</v>
+        <v>-0.0434640017374659</v>
       </c>
     </row>
     <row r="11">
@@ -27036,7 +27036,7 @@
         <v>522</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>-0.0732862388760376</v>
+        <v>-0.0585074030364121</v>
       </c>
     </row>
     <row r="12">
@@ -27044,7 +27044,7 @@
         <v>523</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>-0.0349728899023352</v>
+        <v>-0.0282904299875945</v>
       </c>
     </row>
     <row r="13">
@@ -27052,7 +27052,7 @@
         <v>524</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.0390625584517474</v>
+        <v>0.0330204335605939</v>
       </c>
     </row>
     <row r="14">
@@ -27060,7 +27060,7 @@
         <v>525</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.067626586305301</v>
+        <v>0.0573162432241398</v>
       </c>
     </row>
     <row r="15">
@@ -27068,7 +27068,7 @@
         <v>526</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.0246211747353321</v>
+        <v>0.0187499284528989</v>
       </c>
     </row>
     <row r="16">
@@ -27076,7 +27076,7 @@
         <v>527</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>-0.0179279431371343</v>
+        <v>-0.0154467670968246</v>
       </c>
     </row>
     <row r="17">
@@ -27084,7 +27084,7 @@
         <v>528</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>-0.0344060592248213</v>
+        <v>-0.0264429325743783</v>
       </c>
     </row>
     <row r="18">
@@ -27092,7 +27092,7 @@
         <v>529</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>-0.0349231448214432</v>
+        <v>-0.0304002352173031</v>
       </c>
     </row>
     <row r="19">
@@ -27100,7 +27100,7 @@
         <v>530</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>-0.002698720716451</v>
+        <v>-0.00361378577183889</v>
       </c>
     </row>
     <row r="20">
@@ -27108,7 +27108,7 @@
         <v>531</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.019235451068084</v>
+        <v>0.0240654974465531</v>
       </c>
     </row>
     <row r="21">
@@ -27116,7 +27116,7 @@
         <v>532</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.0152419159036791</v>
+        <v>0.024827790056195</v>
       </c>
     </row>
     <row r="22">
@@ -27124,7 +27124,7 @@
         <v>533</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.0329642179381988</v>
+        <v>0.0366574344176479</v>
       </c>
     </row>
     <row r="23">
@@ -27132,7 +27132,7 @@
         <v>534</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.0603750680804897</v>
+        <v>0.0601505331301639</v>
       </c>
     </row>
     <row r="24">

</xml_diff>